<commit_message>
Update guidance and replace pov_direct data
Modify Guidance note/comments and resonses.xlsx (updated comments/responses). Remove outdated sample_data/pov_direct3.rds and add sample_data/pov_directv4.rds as the new dataset version.
</commit_message>
<xml_diff>
--- a/Guidance note/comments and resonses.xlsx
+++ b/Guidance note/comments and resonses.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/2e19cae34435d3be/EU_SAE_application_package/Guidance note/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="30" documentId="8_{FF178553-A949-41D6-82DC-6740B52A4A4E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5846AD61-AAAE-4A6E-B9C9-D212C0308C74}"/>
+  <xr:revisionPtr revIDLastSave="39" documentId="8_{FF178553-A949-41D6-82DC-6740B52A4A4E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{DC5E69CE-5600-4CFB-BBA0-8DF2D88EA020}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{31817838-8FDE-420F-9849-85D130BF406F}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="35">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="32">
   <si>
     <t>1. Benchmarking doesn’t seem to work, as it seems to refer to Spanish dataset, even though they specify Polish data</t>
   </si>
@@ -416,72 +416,6 @@
   </si>
   <si>
     <r>
-      <t>Welfare typo crashes</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">: confirmed likely cause. </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Arial Unicode MS"/>
-      </rPr>
-      <t>load_and_harmonize()</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> silently skips a missing welfare column instead of erroring; readiness then later uses </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Arial Unicode MS"/>
-      </rPr>
-      <t>survey_data$welfare</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>. Required mapped columns should be validated immediately.</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t>Selecting MFH2 still outputs MFH1</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>: expected current behavior, though confusing. The MFH script always fits MFH1 and MFH2; the “Diagnostic model” only chooses which variant drives downstream diagnostics/reporting. See [scripts/02_mfh.R (line 1153)](C:/Users/noboy/OneDrive/EU_SAE_application_package/scripts/02_mfh.R:1153).</t>
-    </r>
-  </si>
-  <si>
-    <r>
       <t>Benchmark outputs without asking</t>
     </r>
     <r>
@@ -494,90 +428,6 @@
       </rPr>
       <t>: same root cause as #1. Internal benchmark targets are computed from direct estimates when no external benchmark file is given. Point estimates may barely change, while MSE changes because benchmarked MSE is recomputed.</t>
     </r>
-  </si>
-  <si>
-    <r>
-      <t>Strata in sampling variances</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">: not currently supported. Both UFH and MFH use </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Arial Unicode MS"/>
-      </rPr>
-      <t>svydesign(ids = ~psu, weights = ~weight, ...)</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> with no </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Arial Unicode MS"/>
-      </rPr>
-      <t>strata</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">. It can be added via a strata variable mapping and </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Arial Unicode MS"/>
-      </rPr>
-      <t>svydesign(..., strata = ~strata, nest = TRUE)</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>.</t>
-    </r>
-  </si>
-  <si>
-    <t>If they run the models in this way, they first obtained the results of 2019 and 2020, then 2020 and 2021, then 2021 and 2022, and lastly 2022 and 2023. The comment says that some years do not have any poverty rates?</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Using RMSE and point estimates, we can check whether CV is correct. </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Typos should be spotted in the data readiness stage. If there are errors, the errors should be mentioned and prevent users from moving to the analysis stage. </t>
-  </si>
-  <si>
-    <t>Yes. But, the comparison does not include MFH1 analysis. Is this a problem?</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Let's include it. </t>
   </si>
   <si>
     <r>
@@ -594,6 +444,111 @@
 If no population file is uploaded, estimate domain populations from the survey as sum(weight * household size).
 If neither is possible, stop/warn clearly instead of using old sample data.</t>
     </r>
+  </si>
+  <si>
+    <r>
+      <t>Welfare typo crashes</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">: Typos should be spotted in the data readiness stage. If there are errors, the errors should be mentioned and prevent users from moving to the analysis stage. </t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>Selecting MFH2 still outputs MFH1</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>: Modify the code so that the results of only selected one (MFH1, MFH2, or MFH3) will be presented.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>Strata in sampling variances</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">: not currently supported. Both UFH and MFH use </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>svydesign(ids = ~psu, weights = ~weight, ...)</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> with no </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>strata</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">. Let's add a strata variable mapping and </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>svydesign(..., strata = ~strata, nest = TRUE)</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>.</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">15. There is no selection of the level of benchmarking in the dashboard. For example, users should be able to choose the level of benchmarking as national or region. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Include a quesiton on the level of benchmarking in the dashboard. This should be allowed even if users do not provide the benchmarking target database. The app will produce poverty estimates at the level selected for benchmarking using the household survey data. </t>
   </si>
 </sst>
 </file>
@@ -1053,157 +1008,139 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{274E5688-76D1-42B0-94A3-0EF648E39427}">
-  <dimension ref="A1:C15"/>
+  <dimension ref="A1:B16"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
     <col min="1" max="1" width="65.81640625" style="1" customWidth="1"/>
-    <col min="2" max="2" width="51.6328125" style="1" customWidth="1"/>
-    <col min="3" max="3" width="75.08984375" style="1" customWidth="1"/>
+    <col min="2" max="2" width="75.08984375" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3">
+    <row r="1" spans="1:2">
       <c r="A1" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="B1" s="2"/>
-      <c r="C1" s="3" t="s">
+      <c r="B1" s="3" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="2" spans="1:3" ht="58">
+    <row r="2" spans="1:2" ht="58">
       <c r="A2" s="7" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="7"/>
-      <c r="C2" s="8" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" ht="72.5">
+      <c r="B2" s="8" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" ht="72.5">
       <c r="A3" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="4"/>
-      <c r="C3" s="5" t="s">
+      <c r="B3" s="5" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="4" spans="1:3" ht="43.5">
+    <row r="4" spans="1:2" ht="43.5">
       <c r="A4" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="4"/>
-      <c r="C4" s="5" t="s">
+      <c r="B4" s="5" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="5" spans="1:3" ht="58">
+    <row r="5" spans="1:2" ht="58">
       <c r="A5" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="B5" s="4"/>
-      <c r="C5" s="5" t="s">
+      <c r="B5" s="5" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="6" spans="1:3" ht="72.5">
+    <row r="6" spans="1:2" ht="72.5">
       <c r="A6" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="B6" s="4"/>
-      <c r="C6" s="5" t="s">
+      <c r="B6" s="5" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="7" spans="1:3" ht="58">
+    <row r="7" spans="1:2" ht="58">
       <c r="A7" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="B7" s="4"/>
-      <c r="C7" s="5" t="s">
+      <c r="B7" s="5" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="8" spans="1:3" ht="58">
+    <row r="8" spans="1:2" ht="58">
       <c r="A8" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="B8" s="7" t="s">
-        <v>29</v>
-      </c>
-      <c r="C8" s="5" t="s">
+      <c r="B8" s="5" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="9" spans="1:3" ht="58">
+    <row r="9" spans="1:2" ht="58">
       <c r="A9" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="B9" s="4" t="s">
-        <v>30</v>
-      </c>
-      <c r="C9" s="6" t="s">
+      <c r="B9" s="6" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="10" spans="1:3" ht="87">
+    <row r="10" spans="1:2" ht="87">
       <c r="A10" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="B10" s="4"/>
-      <c r="C10" s="5" t="s">
+      <c r="B10" s="5" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="11" spans="1:3" ht="43.5">
+    <row r="11" spans="1:2" ht="43.5">
       <c r="A11" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="B11" s="4"/>
-      <c r="C11" s="5" t="s">
+      <c r="B11" s="5" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="12" spans="1:3" ht="87">
+    <row r="12" spans="1:2" ht="87">
       <c r="A12" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="B12" s="4" t="s">
-        <v>31</v>
-      </c>
-      <c r="C12" s="5" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="13" spans="1:3" ht="58">
+      <c r="B12" s="5" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" ht="29">
       <c r="A13" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="B13" s="4" t="s">
-        <v>32</v>
-      </c>
-      <c r="C13" s="5" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="14" spans="1:3" ht="58">
+      <c r="B13" s="5" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" ht="58">
       <c r="A14" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="B14" s="7"/>
-      <c r="C14" s="5" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="15" spans="1:3" ht="43.5">
+      <c r="B14" s="5" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" ht="43.5">
       <c r="A15" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="B15" s="4" t="s">
-        <v>33</v>
-      </c>
-      <c r="C15" s="5" t="s">
-        <v>28</v>
+      <c r="B15" s="5" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" ht="43.5">
+      <c r="A16" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="B16" s="1" t="s">
+        <v>31</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Use population_weight = weight * hh_size
Compute and use population_weight = weight * hh_size for direct (UFH/MFH) estimates across the app. Added sae_add_population_weight helper and integrated population-weighted logic into validation, diagnostics, UI text, and estimation code (R/validation_checks.R, app.R, app_support.R, scripts/*). Made comparison step more robust (dynamic years, geometry/path handling, domain cleaning, plotting loops) and improved outputs file existence reporting. Removed unused outputs/figures/.gitkeep.
</commit_message>
<xml_diff>
--- a/Guidance note/comments and resonses.xlsx
+++ b/Guidance note/comments and resonses.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/2e19cae34435d3be/EU_SAE_application_package/Guidance note/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="39" documentId="8_{FF178553-A949-41D6-82DC-6740B52A4A4E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{DC5E69CE-5600-4CFB-BBA0-8DF2D88EA020}"/>
+  <xr:revisionPtr revIDLastSave="54" documentId="8_{FF178553-A949-41D6-82DC-6740B52A4A4E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{320AAB7F-0368-452C-8960-8902632E4BBB}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{31817838-8FDE-420F-9849-85D130BF406F}"/>
   </bookViews>
@@ -141,17 +141,47 @@
   </si>
   <si>
     <r>
-      <t>NUTS2/region required</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">: currently yes in practice. The code calls it </t>
+      <t>Wrong analysis year typo</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>: confirmed gap. The app checks “exactly two years” and whether survey/auxiliary contain the same year column, but it does not block requested years that are absent from the data. That should become a clear readiness error.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>2012/2013 labels</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>: confirmed. Several Comparison calls and titles are hard-coded to 2012/2013. See [scripts/03_comparison.R (line 859)](C:/Users/noboy/OneDrive/EU_SAE_application_package/scripts/03_comparison.R:859) and [scripts/03_comparison.R (line 1106)](C:/Users/noboy/OneDrive/EU_SAE_application_package/scripts/03_comparison.R:1106).</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>Province/domain as string with leading zeroes</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">: not safe today. MFH/Comparison repeatedly coerce </t>
     </r>
     <r>
       <rPr>
@@ -159,17 +189,77 @@
         <color theme="1"/>
         <rFont val="Arial Unicode MS"/>
       </rPr>
-      <t>region</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">; because benchmarking is on by default, UFH unconditionally builds </t>
+      <t>domain</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> to integer, which will drop leading zeroes. This should be changed to character IDs throughout joins, maps, benchmark, and exports.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>Benchmark outputs without asking</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>: same root cause as #1. Internal benchmark targets are computed from direct estimates when no external benchmark file is given. Point estimates may barely change, while MSE changes because benchmarked MSE is recomputed.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>Welfare typo crashes</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">: Typos should be spotted in the data readiness stage. If there are errors, the errors should be mentioned and prevent users from moving to the analysis stage. </t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>Selecting MFH2 still outputs MFH1</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>: Modify the code so that the results of only selected one (MFH1, MFH2, or MFH3) will be presented.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>Strata in sampling variances</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">: not currently supported. Both UFH and MFH use </t>
     </r>
     <r>
       <rPr>
@@ -177,32 +267,17 @@
         <color theme="1"/>
         <rFont val="Arial Unicode MS"/>
       </rPr>
-      <t>region_map &lt;- survey_all |&gt; select(domain, region)</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>. This should only be required when benchmarking is enabled.</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t>Run labels/output folders</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">: currently outputs are fixed under </t>
+      <t>svydesign(ids = ~psu, weights = ~weight, ...)</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> with no </t>
     </r>
     <r>
       <rPr>
@@ -210,17 +285,17 @@
         <color theme="1"/>
         <rFont val="Arial Unicode MS"/>
       </rPr>
-      <t>outputs/</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> and overwritten. The app does create timestamped </t>
+      <t>strata</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">. Let's add a strata variable mapping and </t>
     </r>
     <r>
       <rPr>
@@ -228,206 +303,24 @@
         <color theme="1"/>
         <rFont val="Arial Unicode MS"/>
       </rPr>
-      <t>app_runs/&lt;run_id&gt;/</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> folders, but only for config/logs, not the result files. A run label or per-run output folder would be a good fix.</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t>Wrong analysis year typo</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>: confirmed gap. The app checks “exactly two years” and whether survey/auxiliary contain the same year column, but it does not block requested years that are absent from the data. That should become a clear readiness error.</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t>Cannot remove benchmark file</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">: true for the current UI. Once Shiny </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Arial Unicode MS"/>
-      </rPr>
-      <t>fileInput</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> has a file, there is no reset/ignore control here. Add a “Use benchmarking file” checkbox or “Clear benchmark file” button.</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t>Some year pairs produce empty files</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>: likely caused by missing/empty filtered data, unusable variances, or model failures that write placeholder/empty outputs instead of stopping early with a clear message. The checks should assert non-empty rows for both selected years before fitting.</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t>sm_all</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> large MFH CVs</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">: plausible from the code. MFH replaces all sampling variances under </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Arial Unicode MS"/>
-      </rPr>
-      <t>sm_all</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">, builds covariances from those smoothed variances, then CV is </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Arial Unicode MS"/>
-      </rPr>
-      <t>sqrt(MSE) / estimate</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>; if MFH estimates are near zero or smoothed variances inflate, CV can explode. Need the specific output/log to diagnose fully.</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t>2012/2013 labels</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>: confirmed. Several Comparison calls and titles are hard-coded to 2012/2013. See [scripts/03_comparison.R (line 859)](C:/Users/noboy/OneDrive/EU_SAE_application_package/scripts/03_comparison.R:859) and [scripts/03_comparison.R (line 1106)](C:/Users/noboy/OneDrive/EU_SAE_application_package/scripts/03_comparison.R:1106).</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t>Province/domain as string with leading zeroes</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">: not safe today. MFH/Comparison repeatedly coerce </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Arial Unicode MS"/>
-      </rPr>
-      <t>domain</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> to integer, which will drop leading zeroes. This should be changed to character IDs throughout joins, maps, benchmark, and exports.</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t>Benchmark outputs without asking</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>: same root cause as #1. Internal benchmark targets are computed from direct estimates when no external benchmark file is given. Point estimates may barely change, while MSE changes because benchmarked MSE is recomputed.</t>
-    </r>
+      <t>svydesign(..., strata = ~strata, nest = TRUE)</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>.</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">15. There is no selection of the level of benchmarking in the dashboard. For example, users should be able to choose the level of benchmarking as national or region. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Include a quesiton on the level of benchmarking in the dashboard. This should be allowed even if users do not provide the benchmarking target database. The app will produce poverty estimates at the level selected for benchmarking using the household survey data. </t>
   </si>
   <si>
     <r>
@@ -440,54 +333,30 @@
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
-      <t>: Modifications: If a population file is uploaded, use it.
+      <t>: Modifications: First, the dashboard asks users whether they want to include benchmarking. If they say no, benchmarking will not be conducted. If they say yes and  the benchmarking target dataset is uploaded, use it to conduct benchmarking. If they say yes but the target dataset is not provided, the benchmarked datasets will be produced using the household survey data with the level of benchmark selected in the dashboard. 
 If no population file is uploaded, estimate domain populations from the survey as sum(weight * household size).
 If neither is possible, stop/warn clearly instead of using old sample data.</t>
     </r>
   </si>
   <si>
-    <r>
-      <t>Welfare typo crashes</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">: Typos should be spotted in the data readiness stage. If there are errors, the errors should be mentioned and prevent users from moving to the analysis stage. </t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t>Selecting MFH2 still outputs MFH1</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>: Modify the code so that the results of only selected one (MFH1, MFH2, or MFH3) will be presented.</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t>Strata in sampling variances</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">: not currently supported. Both UFH and MFH use </t>
+    <t xml:space="preserve">This issue can be solved by adding the option of benchmarking in the dashboard. </t>
+  </si>
+  <si>
+    <t>Clarification is needed.</t>
+  </si>
+  <si>
+    <r>
+      <t>NUTS2/region required</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">: currently yes in practice. The code calls it </t>
     </r>
     <r>
       <rPr>
@@ -495,17 +364,17 @@
         <color theme="1"/>
         <rFont val="Arial Unicode MS"/>
       </rPr>
-      <t>svydesign(ids = ~psu, weights = ~weight, ...)</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> with no </t>
+      <t>region</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">; because benchmarking is on by default, UFH unconditionally builds </t>
     </r>
     <r>
       <rPr>
@@ -513,17 +382,53 @@
         <color theme="1"/>
         <rFont val="Arial Unicode MS"/>
       </rPr>
-      <t>strata</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">. Let's add a strata variable mapping and </t>
+      <t>region_map &lt;- survey_all |&gt; select(domain, region)</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">. </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>This should only be required when benchmarking is enabled</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>Run labels/output folders</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">: currently outputs are fixed under </t>
     </r>
     <r>
       <rPr>
@@ -531,31 +436,44 @@
         <color theme="1"/>
         <rFont val="Arial Unicode MS"/>
       </rPr>
-      <t>svydesign(..., strata = ~strata, nest = TRUE)</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>.</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">15. There is no selection of the level of benchmarking in the dashboard. For example, users should be able to choose the level of benchmarking as national or region. </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Include a quesiton on the level of benchmarking in the dashboard. This should be allowed even if users do not provide the benchmarking target database. The app will produce poverty estimates at the level selected for benchmarking using the household survey data. </t>
+      <t>outputs/</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> and overwritten. Please save output folders whenever you complete an analysis. </t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>Identification of sources of high CVs</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t xml:space="preserve">. pov_mfh.xlsx and pov_fh.xlsx include all the information to examine why CV is so high (too high RMSE or too low point estimate). Both are vailable in output/data folder. </t>
+    </r>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="9">
+  <fonts count="10">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -614,6 +532,11 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <name val="Aptos"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -650,7 +573,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -665,13 +588,22 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1023,11 +955,11 @@
         <v>15</v>
       </c>
     </row>
-    <row r="2" spans="1:2" ht="58">
-      <c r="A2" s="7" t="s">
+    <row r="2" spans="1:2" ht="116">
+      <c r="A2" s="8" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="8" t="s">
+      <c r="B2" s="7" t="s">
         <v>26</v>
       </c>
     </row>
@@ -1044,7 +976,7 @@
         <v>2</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>17</v>
+        <v>29</v>
       </c>
     </row>
     <row r="5" spans="1:2" ht="58">
@@ -1052,7 +984,7 @@
         <v>3</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>18</v>
+        <v>30</v>
       </c>
     </row>
     <row r="6" spans="1:2" ht="72.5">
@@ -1060,31 +992,31 @@
         <v>4</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
     </row>
     <row r="7" spans="1:2" ht="58">
       <c r="A7" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="B7" s="5" t="s">
-        <v>20</v>
+      <c r="B7" s="11" t="s">
+        <v>27</v>
       </c>
     </row>
     <row r="8" spans="1:2" ht="58">
-      <c r="A8" s="7" t="s">
+      <c r="A8" s="6" t="s">
         <v>6</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="9" spans="1:2" ht="58">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" ht="42">
       <c r="A9" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="B9" s="6" t="s">
-        <v>22</v>
+      <c r="B9" s="10" t="s">
+        <v>31</v>
       </c>
     </row>
     <row r="10" spans="1:2" ht="87">
@@ -1092,7 +1024,7 @@
         <v>8</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>23</v>
+        <v>18</v>
       </c>
     </row>
     <row r="11" spans="1:2" ht="43.5">
@@ -1100,7 +1032,7 @@
         <v>9</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>24</v>
+        <v>19</v>
       </c>
     </row>
     <row r="12" spans="1:2" ht="87">
@@ -1108,7 +1040,7 @@
         <v>10</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>27</v>
+        <v>21</v>
       </c>
     </row>
     <row r="13" spans="1:2" ht="29">
@@ -1116,15 +1048,15 @@
         <v>11</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>28</v>
+        <v>22</v>
       </c>
     </row>
     <row r="14" spans="1:2" ht="58">
-      <c r="A14" s="7" t="s">
+      <c r="A14" s="6" t="s">
         <v>12</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>25</v>
+        <v>20</v>
       </c>
     </row>
     <row r="15" spans="1:2" ht="43.5">
@@ -1132,15 +1064,15 @@
         <v>13</v>
       </c>
       <c r="B15" s="5" t="s">
-        <v>29</v>
+        <v>23</v>
       </c>
     </row>
     <row r="16" spans="1:2" ht="43.5">
-      <c r="A16" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="B16" s="1" t="s">
-        <v>31</v>
+      <c r="A16" s="9" t="s">
+        <v>24</v>
+      </c>
+      <c r="B16" s="9" t="s">
+        <v>25</v>
       </c>
     </row>
   </sheetData>

</xml_diff>